<commit_message>
cover_nan_0224_age_IVFDI.py: df_DI와 df_IVF에서 값의 종류가 1개인 컬럼들 삭제
</commit_message>
<xml_diff>
--- a/shared codes/data/데이터 명세.xlsx
+++ b/shared codes/data/데이터 명세.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/downy/Documents/2025 LG aimers/DKU-LG-Capstone-6/shared codes/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64021AB-B4AE-7948-91D8-17A329256B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320D0073-E7B0-EF41-885D-0233D3798AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{DA19DC8F-9B0C-4123-9D80-76730E032BF2}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{DA19DC8F-9B0C-4123-9D80-76730E032BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="데이터 명세" sheetId="1" r:id="rId1"/>

</xml_diff>